<commit_message>
Successfully Writing to Rad Archive Sheet and updated template
Working on writing to printout next
</commit_message>
<xml_diff>
--- a/Python_Scripts/Radioligand_Binding/data_files/Radioactivity_Archive_Template.xlsx
+++ b/Python_Scripts/Radioligand_Binding/data_files/Radioactivity_Archive_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tlalbert\Documents\PDSP\Python_Scripts\Radioligand_Binding\data_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tlalbert\Documents\PDSP_rewrite\Python_Scripts\Radioligand_Binding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A14DD49-9542-4CFA-A8F1-13F500215B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E2F1BFC-BA57-4BDF-8E86-9F96A2E3AD95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4005" yWindow="2790" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9015" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Binding Type</t>
   </si>
@@ -68,49 +68,10 @@
     <t>Receptor</t>
   </si>
   <si>
-    <t>Specific Activity (Ci/mmol)</t>
-  </si>
-  <si>
     <t>Assay Conc. (nM)</t>
   </si>
   <si>
     <t>Actual Assay Conc. (nM)</t>
-  </si>
-  <si>
-    <t>Reference</t>
-  </si>
-  <si>
-    <t>Number of Plates</t>
-  </si>
-  <si>
-    <t>Number of Pellets</t>
-  </si>
-  <si>
-    <t>Buffer Volume (mL)</t>
-  </si>
-  <si>
-    <t>Ligand Volume (µL)</t>
-  </si>
-  <si>
-    <t>uCi/uL Ligand Ratio</t>
-  </si>
-  <si>
-    <t>uCi</t>
-  </si>
-  <si>
-    <t>Sink Disposal (80%) (uCi)</t>
-  </si>
-  <si>
-    <t>Dry Waste (20%) (uCi)</t>
-  </si>
-  <si>
-    <t>Assay BB</t>
-  </si>
-  <si>
-    <t>PRIM Pellet/Plate</t>
-  </si>
-  <si>
-    <t>SEC Pellet/Plate</t>
   </si>
   <si>
     <t>Ligand</t>
@@ -121,6 +82,84 @@
   </si>
   <si>
     <t>Inventory Control Number</t>
+  </si>
+  <si>
+    <t>Specific Activity (Ci/mmol)</t>
+  </si>
+  <si>
+    <t>Initial Quantity (mCi)</t>
+  </si>
+  <si>
+    <t>Initial Volume (uL)</t>
+  </si>
+  <si>
+    <t>uCi/uL Ligand Ratio</t>
+  </si>
+  <si>
+    <t>mCi Remaining</t>
+  </si>
+  <si>
+    <t>uL Remaining</t>
+  </si>
+  <si>
+    <t>Date Received</t>
+  </si>
+  <si>
+    <t>Date Started</t>
+  </si>
+  <si>
+    <t>Date Last Used</t>
+  </si>
+  <si>
+    <t>Calibration Date</t>
+  </si>
+  <si>
+    <t>Decay Factor</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>Number of Plates</t>
+  </si>
+  <si>
+    <t>Number of Pellets</t>
+  </si>
+  <si>
+    <t>Buffer Volume (mL)</t>
+  </si>
+  <si>
+    <t>Ligand Volume (µL)</t>
+  </si>
+  <si>
+    <t>uCi</t>
+  </si>
+  <si>
+    <t>Sink Disposal (80%) (uCi)</t>
+  </si>
+  <si>
+    <t>Dry Waste (20%) (uCi)</t>
+  </si>
+  <si>
+    <t>Assay BB</t>
+  </si>
+  <si>
+    <t>Filter Type</t>
+  </si>
+  <si>
+    <t>Unifilter Pellet Ratio</t>
+  </si>
+  <si>
+    <t>Filtermat Pellet Ratio</t>
+  </si>
+  <si>
+    <t>Pellets in Inventory</t>
+  </si>
+  <si>
+    <t>Assay DB Notes</t>
+  </si>
+  <si>
+    <t>Pellet DB Notes</t>
   </si>
 </sst>
 </file>
@@ -523,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI1"/>
+  <dimension ref="A1:AV1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
@@ -536,21 +575,34 @@
     <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="3.28515625" customWidth="1"/>
+    <col min="13" max="13" width="1.7109375" customWidth="1"/>
+    <col min="14" max="14" width="2.28515625" customWidth="1"/>
+    <col min="15" max="15" width="2" customWidth="1"/>
     <col min="17" max="17" width="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.7109375" customWidth="1"/>
-    <col min="20" max="20" width="14.5703125" customWidth="1"/>
-    <col min="21" max="21" width="10" customWidth="1"/>
-    <col min="24" max="24" width="9.85546875" customWidth="1"/>
-    <col min="29" max="29" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.42578125" customWidth="1"/>
-    <col min="32" max="32" width="11.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="7.140625" customWidth="1"/>
-    <col min="35" max="35" width="7.28515625" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" customWidth="1"/>
+    <col min="20" max="20" width="16.85546875" customWidth="1"/>
+    <col min="21" max="21" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.140625" customWidth="1"/>
+    <col min="26" max="26" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.42578125" customWidth="1"/>
+    <col min="28" max="28" width="10.5703125" customWidth="1"/>
+    <col min="29" max="29" width="11.85546875" customWidth="1"/>
+    <col min="30" max="30" width="12" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" customWidth="1"/>
+    <col min="32" max="32" width="10.5703125" customWidth="1"/>
+    <col min="33" max="33" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.42578125" customWidth="1"/>
+    <col min="35" max="35" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="11.42578125" customWidth="1"/>
+    <col min="41" max="41" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:48" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -591,58 +643,97 @@
         <v>10</v>
       </c>
       <c r="R1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="AG1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="AH1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="U1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="AG1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AI1" s="2" t="s">
-        <v>25</v>
+      <c r="AJ1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AL1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AM1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AN1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AO1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AP1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AQ1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AU1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AV1" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating templates, and schema, ready to write to binding printout
</commit_message>
<xml_diff>
--- a/Python_Scripts/Radioligand_Binding/data_files/Radioactivity_Archive_Template.xlsx
+++ b/Python_Scripts/Radioligand_Binding/data_files/Radioactivity_Archive_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tlalbert\Documents\PDSP_rewrite\Python_Scripts\Radioligand_Binding\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tlalbert\Documents\PDSP_rewrite\Python_Scripts\Radioligand_Binding\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E2F1BFC-BA57-4BDF-8E86-9F96A2E3AD95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50851450-400A-4FF2-80F6-A78B691F3371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9015" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Binding Type</t>
   </si>
@@ -102,12 +102,6 @@
     <t>uL Remaining</t>
   </si>
   <si>
-    <t>Date Received</t>
-  </si>
-  <si>
-    <t>Date Started</t>
-  </si>
-  <si>
     <t>Date Last Used</t>
   </si>
   <si>
@@ -160,6 +154,15 @@
   </si>
   <si>
     <t>Pellet DB Notes</t>
+  </si>
+  <si>
+    <t>Pellet Used</t>
+  </si>
+  <si>
+    <t>Date Received Ligand</t>
+  </si>
+  <si>
+    <t>Date Started Ligand</t>
   </si>
 </sst>
 </file>
@@ -562,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AV1"/>
+  <dimension ref="A1:AW1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
@@ -580,29 +583,30 @@
     <col min="15" max="15" width="2" customWidth="1"/>
     <col min="17" max="17" width="9" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="10.85546875" customWidth="1"/>
-    <col min="20" max="20" width="16.85546875" customWidth="1"/>
-    <col min="21" max="21" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.140625" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.42578125" customWidth="1"/>
-    <col min="28" max="28" width="10.5703125" customWidth="1"/>
-    <col min="29" max="29" width="11.85546875" customWidth="1"/>
-    <col min="30" max="30" width="12" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" customWidth="1"/>
-    <col min="32" max="32" width="10.5703125" customWidth="1"/>
-    <col min="33" max="33" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.42578125" customWidth="1"/>
-    <col min="35" max="35" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="11.42578125" customWidth="1"/>
-    <col min="41" max="41" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="9.85546875" customWidth="1"/>
+    <col min="20" max="20" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.85546875" customWidth="1"/>
+    <col min="22" max="22" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.140625" customWidth="1"/>
+    <col min="27" max="27" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="10.42578125" customWidth="1"/>
+    <col min="29" max="29" width="10.5703125" customWidth="1"/>
+    <col min="30" max="30" width="11.85546875" customWidth="1"/>
+    <col min="31" max="31" width="12" customWidth="1"/>
+    <col min="32" max="32" width="11.5703125" customWidth="1"/>
+    <col min="33" max="33" width="10.5703125" customWidth="1"/>
+    <col min="34" max="34" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.42578125" customWidth="1"/>
+    <col min="36" max="36" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11.42578125" customWidth="1"/>
+    <col min="42" max="42" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -649,91 +653,94 @@
         <v>12</v>
       </c>
       <c r="T1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="U1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AN1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AO1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AP1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="AR1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AU1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AV1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AW1" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="AU1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="AV1" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>